<commit_message>
Upd Incremento 2 Main File
</commit_message>
<xml_diff>
--- a/documentation/Grupo 2 - Organización Trabajo.xlsx
+++ b/documentation/Grupo 2 - Organización Trabajo.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="84">
   <si>
     <t>F</t>
   </si>
@@ -208,9 +208,6 @@
     <t>Diagramas de Secuencia</t>
   </si>
   <si>
-    <t>Pendiente</t>
-  </si>
-  <si>
     <t>Actualización Diagramas</t>
   </si>
   <si>
@@ -220,10 +217,52 @@
     <t>Francisco Torres , Bastian Benítez</t>
   </si>
   <si>
+    <t>Bastian Benítez, Francisco Torres</t>
+  </si>
+  <si>
     <t>Composición Documento Incremento 2</t>
   </si>
   <si>
+    <t>Samir Saud, Manuel Vidal , Gerónimo Lopez, Francisco Torres, Eliam Rivas , Bastian Benítez</t>
+  </si>
+  <si>
     <t>Recorrecion Documento 0 e Incremento 1</t>
+  </si>
+  <si>
+    <t>Incremento 3</t>
+  </si>
+  <si>
+    <t>Eliam Rivas , Manuel Vidal</t>
+  </si>
+  <si>
+    <t>Eliam Rivas , Francisco Torres</t>
+  </si>
+  <si>
+    <t>Bastian Benítez , Gerónimo Lopez, Manuel Vidal , Samir Saud</t>
+  </si>
+  <si>
+    <t>Eliam Rivas, Francisco Torres , Bastian Benítez</t>
+  </si>
+  <si>
+    <t>Gerónimo Lopez, Manuel Vidal , Samir Saud, Eliam Rivas</t>
+  </si>
+  <si>
+    <t>Creación de Videos de Documentación</t>
+  </si>
+  <si>
+    <t>Bastian Benítez , Gerónimo Lopez, Manuel Vidal , Samir Saud, Eliam Rivas</t>
+  </si>
+  <si>
+    <t>Composición Documento Incremento 3</t>
+  </si>
+  <si>
+    <t>Francisco Torres, Eliam Rivas</t>
+  </si>
+  <si>
+    <t>Bastian Benítez , Manuel Vidal</t>
+  </si>
+  <si>
+    <t>Recorrecion Documento 0,Incremento 1 y 2</t>
   </si>
 </sst>
 </file>
@@ -1072,12 +1111,12 @@
         <v>60</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>65</v>
+        <v>8</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B40" s="7" t="s">
         <v>39</v>
@@ -1086,7 +1125,7 @@
         <v>60</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>65</v>
+        <v>8</v>
       </c>
     </row>
     <row r="41">
@@ -1094,10 +1133,10 @@
         <v>52</v>
       </c>
       <c r="B41" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="C41" s="8" t="s">
         <v>67</v>
-      </c>
-      <c r="C41" s="8" t="s">
-        <v>68</v>
       </c>
       <c r="D41" s="6" t="s">
         <v>8</v>
@@ -1107,98 +1146,211 @@
       <c r="A42" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B42" s="7"/>
-      <c r="C42" s="11"/>
+      <c r="B42" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="C42" s="8" t="s">
+        <v>67</v>
+      </c>
       <c r="D42" s="6" t="s">
-        <v>65</v>
+        <v>8</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="B43" s="7"/>
-      <c r="C43" s="11"/>
+      <c r="B43" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="C43" s="8" t="s">
+        <v>68</v>
+      </c>
       <c r="D43" s="6" t="s">
-        <v>65</v>
+        <v>8</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="B44" s="7"/>
-      <c r="C44" s="11"/>
+      <c r="B44" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="C44" s="8" t="s">
+        <v>39</v>
+      </c>
       <c r="D44" s="6" t="s">
-        <v>65</v>
+        <v>8</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B45" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C45" s="11"/>
+      <c r="C45" s="8" t="s">
+        <v>39</v>
+      </c>
       <c r="D45" s="6" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="46">
-      <c r="B46" s="12"/>
-      <c r="C46" s="11"/>
-      <c r="D46" s="11"/>
+      <c r="A46" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="B46" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="47">
-      <c r="B47" s="12"/>
-      <c r="C47" s="11"/>
-      <c r="D47" s="11"/>
+      <c r="A47" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B47" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C47" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="D47" s="6" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="48">
-      <c r="B48" s="12"/>
-      <c r="C48" s="11"/>
-      <c r="D48" s="11"/>
+      <c r="A48" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B48" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="C48" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="D48" s="6" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="49">
-      <c r="B49" s="12"/>
-      <c r="C49" s="11"/>
-      <c r="D49" s="11"/>
+      <c r="A49" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="B49" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="C49" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D49" s="6" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="50">
-      <c r="B50" s="12"/>
-      <c r="C50" s="11"/>
-      <c r="D50" s="11"/>
+      <c r="A50" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="B50" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C50" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="D50" s="6" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="51">
-      <c r="B51" s="12"/>
-      <c r="C51" s="11"/>
-      <c r="D51" s="11"/>
+      <c r="A51" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B51" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C51" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="D51" s="6" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="52">
-      <c r="B52" s="12"/>
-      <c r="C52" s="11"/>
-      <c r="D52" s="11"/>
+      <c r="A52" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B52" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="C52" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D52" s="6" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="53">
-      <c r="B53" s="2"/>
-      <c r="C53" s="11"/>
-      <c r="D53" s="11"/>
+      <c r="A53" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B53" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="C53" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D53" s="6" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="54">
-      <c r="B54" s="2"/>
-      <c r="C54" s="11"/>
-      <c r="D54" s="11"/>
+      <c r="A54" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B54" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="C54" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="D54" s="6" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="55">
-      <c r="B55" s="7"/>
-      <c r="C55" s="11"/>
-      <c r="D55" s="11"/>
+      <c r="A55" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="B55" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="C55" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="D55" s="6" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="56">
-      <c r="B56" s="7"/>
-      <c r="C56" s="11"/>
-      <c r="D56" s="11"/>
+      <c r="A56" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="B56" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C56" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="D56" s="6" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="57">
       <c r="B57" s="7"/>
@@ -1226,7 +1378,7 @@
       <c r="D61" s="11"/>
     </row>
     <row r="62">
-      <c r="B62" s="7"/>
+      <c r="B62" s="12"/>
       <c r="C62" s="11"/>
       <c r="D62" s="11"/>
     </row>
@@ -1261,7 +1413,7 @@
       <c r="D68" s="11"/>
     </row>
     <row r="69">
-      <c r="B69" s="12"/>
+      <c r="B69" s="2"/>
       <c r="C69" s="11"/>
       <c r="D69" s="11"/>
     </row>
@@ -1271,7 +1423,7 @@
       <c r="D70" s="11"/>
     </row>
     <row r="71">
-      <c r="B71" s="2"/>
+      <c r="B71" s="7"/>
       <c r="C71" s="11"/>
       <c r="D71" s="11"/>
     </row>
@@ -1311,7 +1463,7 @@
       <c r="D78" s="11"/>
     </row>
     <row r="79">
-      <c r="B79" s="7"/>
+      <c r="B79" s="12"/>
       <c r="C79" s="11"/>
       <c r="D79" s="11"/>
     </row>
@@ -1346,7 +1498,7 @@
       <c r="D85" s="11"/>
     </row>
     <row r="86">
-      <c r="B86" s="12"/>
+      <c r="B86" s="2"/>
       <c r="C86" s="11"/>
       <c r="D86" s="11"/>
     </row>
@@ -1356,7 +1508,7 @@
       <c r="D87" s="11"/>
     </row>
     <row r="88">
-      <c r="B88" s="2"/>
+      <c r="B88" s="7"/>
       <c r="C88" s="11"/>
       <c r="D88" s="11"/>
     </row>
@@ -1396,7 +1548,7 @@
       <c r="D95" s="11"/>
     </row>
     <row r="96">
-      <c r="B96" s="7"/>
+      <c r="B96" s="12"/>
       <c r="C96" s="11"/>
       <c r="D96" s="11"/>
     </row>
@@ -1431,7 +1583,7 @@
       <c r="D102" s="11"/>
     </row>
     <row r="103">
-      <c r="B103" s="12"/>
+      <c r="B103" s="2"/>
       <c r="C103" s="11"/>
       <c r="D103" s="11"/>
     </row>
@@ -1441,7 +1593,7 @@
       <c r="D104" s="11"/>
     </row>
     <row r="105">
-      <c r="B105" s="2"/>
+      <c r="B105" s="7"/>
       <c r="C105" s="11"/>
       <c r="D105" s="11"/>
     </row>
@@ -1481,7 +1633,7 @@
       <c r="D112" s="11"/>
     </row>
     <row r="113">
-      <c r="B113" s="7"/>
+      <c r="B113" s="12"/>
       <c r="C113" s="11"/>
       <c r="D113" s="11"/>
     </row>
@@ -1516,7 +1668,7 @@
       <c r="D119" s="11"/>
     </row>
     <row r="120">
-      <c r="B120" s="12"/>
+      <c r="B120" s="2"/>
       <c r="C120" s="11"/>
       <c r="D120" s="11"/>
     </row>
@@ -1526,7 +1678,7 @@
       <c r="D121" s="11"/>
     </row>
     <row r="122">
-      <c r="B122" s="2"/>
+      <c r="B122" s="7"/>
       <c r="C122" s="11"/>
       <c r="D122" s="11"/>
     </row>
@@ -1566,7 +1718,7 @@
       <c r="D129" s="11"/>
     </row>
     <row r="130">
-      <c r="B130" s="7"/>
+      <c r="B130" s="12"/>
       <c r="C130" s="11"/>
       <c r="D130" s="11"/>
     </row>
@@ -1601,7 +1753,7 @@
       <c r="D136" s="11"/>
     </row>
     <row r="137">
-      <c r="B137" s="12"/>
+      <c r="B137" s="2"/>
       <c r="C137" s="11"/>
       <c r="D137" s="11"/>
     </row>
@@ -1611,7 +1763,7 @@
       <c r="D138" s="11"/>
     </row>
     <row r="139">
-      <c r="B139" s="2"/>
+      <c r="B139" s="7"/>
       <c r="C139" s="11"/>
       <c r="D139" s="11"/>
     </row>
@@ -1651,7 +1803,7 @@
       <c r="D146" s="11"/>
     </row>
     <row r="147">
-      <c r="B147" s="7"/>
+      <c r="B147" s="12"/>
       <c r="C147" s="11"/>
       <c r="D147" s="11"/>
     </row>
@@ -1686,7 +1838,7 @@
       <c r="D153" s="11"/>
     </row>
     <row r="154">
-      <c r="B154" s="12"/>
+      <c r="B154" s="2"/>
       <c r="C154" s="11"/>
       <c r="D154" s="11"/>
     </row>
@@ -1696,7 +1848,7 @@
       <c r="D155" s="11"/>
     </row>
     <row r="156">
-      <c r="B156" s="2"/>
+      <c r="B156" s="7"/>
       <c r="C156" s="11"/>
       <c r="D156" s="11"/>
     </row>
@@ -1736,7 +1888,7 @@
       <c r="D163" s="11"/>
     </row>
     <row r="164">
-      <c r="B164" s="7"/>
+      <c r="B164" s="12"/>
       <c r="C164" s="11"/>
       <c r="D164" s="11"/>
     </row>
@@ -1771,7 +1923,7 @@
       <c r="D170" s="11"/>
     </row>
     <row r="171">
-      <c r="B171" s="12"/>
+      <c r="B171" s="2"/>
       <c r="C171" s="11"/>
       <c r="D171" s="11"/>
     </row>
@@ -1781,7 +1933,7 @@
       <c r="D172" s="11"/>
     </row>
     <row r="173">
-      <c r="B173" s="2"/>
+      <c r="B173" s="7"/>
       <c r="C173" s="11"/>
       <c r="D173" s="11"/>
     </row>
@@ -1821,7 +1973,7 @@
       <c r="D180" s="11"/>
     </row>
     <row r="181">
-      <c r="B181" s="7"/>
+      <c r="B181" s="12"/>
       <c r="C181" s="11"/>
       <c r="D181" s="11"/>
     </row>
@@ -1856,7 +2008,7 @@
       <c r="D187" s="11"/>
     </row>
     <row r="188">
-      <c r="B188" s="12"/>
+      <c r="B188" s="2"/>
       <c r="C188" s="11"/>
       <c r="D188" s="11"/>
     </row>
@@ -1866,7 +2018,7 @@
       <c r="D189" s="11"/>
     </row>
     <row r="190">
-      <c r="B190" s="2"/>
+      <c r="B190" s="7"/>
       <c r="C190" s="11"/>
       <c r="D190" s="11"/>
     </row>
@@ -1906,7 +2058,7 @@
       <c r="D197" s="11"/>
     </row>
     <row r="198">
-      <c r="B198" s="7"/>
+      <c r="B198" s="12"/>
       <c r="C198" s="11"/>
       <c r="D198" s="11"/>
     </row>
@@ -1941,7 +2093,7 @@
       <c r="D204" s="11"/>
     </row>
     <row r="205">
-      <c r="B205" s="12"/>
+      <c r="B205" s="2"/>
       <c r="C205" s="11"/>
       <c r="D205" s="11"/>
     </row>
@@ -1951,7 +2103,7 @@
       <c r="D206" s="11"/>
     </row>
     <row r="207">
-      <c r="B207" s="2"/>
+      <c r="B207" s="7"/>
       <c r="C207" s="11"/>
       <c r="D207" s="11"/>
     </row>
@@ -1991,7 +2143,7 @@
       <c r="D214" s="11"/>
     </row>
     <row r="215">
-      <c r="B215" s="7"/>
+      <c r="B215" s="12"/>
       <c r="C215" s="11"/>
       <c r="D215" s="11"/>
     </row>
@@ -2026,7 +2178,7 @@
       <c r="D221" s="11"/>
     </row>
     <row r="222">
-      <c r="B222" s="12"/>
+      <c r="B222" s="2"/>
       <c r="C222" s="11"/>
       <c r="D222" s="11"/>
     </row>
@@ -2036,7 +2188,7 @@
       <c r="D223" s="11"/>
     </row>
     <row r="224">
-      <c r="B224" s="2"/>
+      <c r="B224" s="7"/>
       <c r="C224" s="11"/>
       <c r="D224" s="11"/>
     </row>
@@ -2076,7 +2228,7 @@
       <c r="D231" s="11"/>
     </row>
     <row r="232">
-      <c r="B232" s="7"/>
+      <c r="B232" s="12"/>
       <c r="C232" s="11"/>
       <c r="D232" s="11"/>
     </row>
@@ -2111,7 +2263,7 @@
       <c r="D238" s="11"/>
     </row>
     <row r="239">
-      <c r="B239" s="12"/>
+      <c r="B239" s="2"/>
       <c r="C239" s="11"/>
       <c r="D239" s="11"/>
     </row>
@@ -2121,7 +2273,7 @@
       <c r="D240" s="11"/>
     </row>
     <row r="241">
-      <c r="B241" s="2"/>
+      <c r="B241" s="7"/>
       <c r="C241" s="11"/>
       <c r="D241" s="11"/>
     </row>
@@ -2161,7 +2313,7 @@
       <c r="D248" s="11"/>
     </row>
     <row r="249">
-      <c r="B249" s="7"/>
+      <c r="B249" s="12"/>
       <c r="C249" s="11"/>
       <c r="D249" s="11"/>
     </row>
@@ -2196,7 +2348,7 @@
       <c r="D255" s="11"/>
     </row>
     <row r="256">
-      <c r="B256" s="12"/>
+      <c r="B256" s="2"/>
       <c r="C256" s="11"/>
       <c r="D256" s="11"/>
     </row>
@@ -2206,7 +2358,7 @@
       <c r="D257" s="11"/>
     </row>
     <row r="258">
-      <c r="B258" s="2"/>
+      <c r="B258" s="7"/>
       <c r="C258" s="11"/>
       <c r="D258" s="11"/>
     </row>
@@ -2246,7 +2398,7 @@
       <c r="D265" s="11"/>
     </row>
     <row r="266">
-      <c r="B266" s="7"/>
+      <c r="B266" s="12"/>
       <c r="C266" s="11"/>
       <c r="D266" s="11"/>
     </row>
@@ -2281,7 +2433,7 @@
       <c r="D272" s="11"/>
     </row>
     <row r="273">
-      <c r="B273" s="12"/>
+      <c r="B273" s="2"/>
       <c r="C273" s="11"/>
       <c r="D273" s="11"/>
     </row>
@@ -2291,7 +2443,7 @@
       <c r="D274" s="11"/>
     </row>
     <row r="275">
-      <c r="B275" s="2"/>
+      <c r="B275" s="7"/>
       <c r="C275" s="11"/>
       <c r="D275" s="11"/>
     </row>
@@ -2331,7 +2483,7 @@
       <c r="D282" s="11"/>
     </row>
     <row r="283">
-      <c r="B283" s="7"/>
+      <c r="B283" s="12"/>
       <c r="C283" s="11"/>
       <c r="D283" s="11"/>
     </row>
@@ -2366,7 +2518,7 @@
       <c r="D289" s="11"/>
     </row>
     <row r="290">
-      <c r="B290" s="12"/>
+      <c r="B290" s="2"/>
       <c r="C290" s="11"/>
       <c r="D290" s="11"/>
     </row>
@@ -2376,7 +2528,7 @@
       <c r="D291" s="11"/>
     </row>
     <row r="292">
-      <c r="B292" s="2"/>
+      <c r="B292" s="7"/>
       <c r="C292" s="11"/>
       <c r="D292" s="11"/>
     </row>
@@ -2416,7 +2568,7 @@
       <c r="D299" s="11"/>
     </row>
     <row r="300">
-      <c r="B300" s="7"/>
+      <c r="B300" s="12"/>
       <c r="C300" s="11"/>
       <c r="D300" s="11"/>
     </row>
@@ -2451,7 +2603,7 @@
       <c r="D306" s="11"/>
     </row>
     <row r="307">
-      <c r="B307" s="12"/>
+      <c r="B307" s="2"/>
       <c r="C307" s="11"/>
       <c r="D307" s="11"/>
     </row>
@@ -2461,7 +2613,7 @@
       <c r="D308" s="11"/>
     </row>
     <row r="309">
-      <c r="B309" s="2"/>
+      <c r="B309" s="7"/>
       <c r="C309" s="11"/>
       <c r="D309" s="11"/>
     </row>
@@ -2501,7 +2653,7 @@
       <c r="D316" s="11"/>
     </row>
     <row r="317">
-      <c r="B317" s="7"/>
+      <c r="B317" s="12"/>
       <c r="C317" s="11"/>
       <c r="D317" s="11"/>
     </row>
@@ -2536,7 +2688,7 @@
       <c r="D323" s="11"/>
     </row>
     <row r="324">
-      <c r="B324" s="12"/>
+      <c r="B324" s="2"/>
       <c r="C324" s="11"/>
       <c r="D324" s="11"/>
     </row>
@@ -2546,7 +2698,7 @@
       <c r="D325" s="11"/>
     </row>
     <row r="326">
-      <c r="B326" s="2"/>
+      <c r="B326" s="7"/>
       <c r="C326" s="11"/>
       <c r="D326" s="11"/>
     </row>
@@ -2586,7 +2738,7 @@
       <c r="D333" s="11"/>
     </row>
     <row r="334">
-      <c r="B334" s="7"/>
+      <c r="B334" s="12"/>
       <c r="C334" s="11"/>
       <c r="D334" s="11"/>
     </row>
@@ -2621,7 +2773,7 @@
       <c r="D340" s="11"/>
     </row>
     <row r="341">
-      <c r="B341" s="12"/>
+      <c r="B341" s="2"/>
       <c r="C341" s="11"/>
       <c r="D341" s="11"/>
     </row>
@@ -2631,7 +2783,7 @@
       <c r="D342" s="11"/>
     </row>
     <row r="343">
-      <c r="B343" s="2"/>
+      <c r="B343" s="7"/>
       <c r="C343" s="11"/>
       <c r="D343" s="11"/>
     </row>
@@ -2671,7 +2823,7 @@
       <c r="D350" s="11"/>
     </row>
     <row r="351">
-      <c r="B351" s="7"/>
+      <c r="B351" s="12"/>
       <c r="C351" s="11"/>
       <c r="D351" s="11"/>
     </row>
@@ -2706,7 +2858,7 @@
       <c r="D357" s="11"/>
     </row>
     <row r="358">
-      <c r="B358" s="12"/>
+      <c r="B358" s="2"/>
       <c r="C358" s="11"/>
       <c r="D358" s="11"/>
     </row>
@@ -2716,7 +2868,7 @@
       <c r="D359" s="11"/>
     </row>
     <row r="360">
-      <c r="B360" s="2"/>
+      <c r="B360" s="7"/>
       <c r="C360" s="11"/>
       <c r="D360" s="11"/>
     </row>
@@ -2756,7 +2908,7 @@
       <c r="D367" s="11"/>
     </row>
     <row r="368">
-      <c r="B368" s="7"/>
+      <c r="B368" s="12"/>
       <c r="C368" s="11"/>
       <c r="D368" s="11"/>
     </row>
@@ -2791,7 +2943,7 @@
       <c r="D374" s="11"/>
     </row>
     <row r="375">
-      <c r="B375" s="12"/>
+      <c r="B375" s="2"/>
       <c r="C375" s="11"/>
       <c r="D375" s="11"/>
     </row>
@@ -2801,7 +2953,7 @@
       <c r="D376" s="11"/>
     </row>
     <row r="377">
-      <c r="B377" s="2"/>
+      <c r="B377" s="7"/>
       <c r="C377" s="11"/>
       <c r="D377" s="11"/>
     </row>
@@ -2841,7 +2993,7 @@
       <c r="D384" s="11"/>
     </row>
     <row r="385">
-      <c r="B385" s="7"/>
+      <c r="B385" s="12"/>
       <c r="C385" s="11"/>
       <c r="D385" s="11"/>
     </row>
@@ -2876,7 +3028,7 @@
       <c r="D391" s="11"/>
     </row>
     <row r="392">
-      <c r="B392" s="12"/>
+      <c r="B392" s="2"/>
       <c r="C392" s="11"/>
       <c r="D392" s="11"/>
     </row>
@@ -2886,7 +3038,7 @@
       <c r="D393" s="11"/>
     </row>
     <row r="394">
-      <c r="B394" s="2"/>
+      <c r="B394" s="7"/>
       <c r="C394" s="11"/>
       <c r="D394" s="11"/>
     </row>
@@ -2926,7 +3078,7 @@
       <c r="D401" s="11"/>
     </row>
     <row r="402">
-      <c r="B402" s="7"/>
+      <c r="B402" s="12"/>
       <c r="C402" s="11"/>
       <c r="D402" s="11"/>
     </row>
@@ -2961,7 +3113,7 @@
       <c r="D408" s="11"/>
     </row>
     <row r="409">
-      <c r="B409" s="12"/>
+      <c r="B409" s="2"/>
       <c r="C409" s="11"/>
       <c r="D409" s="11"/>
     </row>
@@ -2971,7 +3123,7 @@
       <c r="D410" s="11"/>
     </row>
     <row r="411">
-      <c r="B411" s="2"/>
+      <c r="B411" s="7"/>
       <c r="C411" s="11"/>
       <c r="D411" s="11"/>
     </row>
@@ -3011,7 +3163,7 @@
       <c r="D418" s="11"/>
     </row>
     <row r="419">
-      <c r="B419" s="7"/>
+      <c r="B419" s="12"/>
       <c r="C419" s="11"/>
       <c r="D419" s="11"/>
     </row>
@@ -3046,7 +3198,7 @@
       <c r="D425" s="11"/>
     </row>
     <row r="426">
-      <c r="B426" s="12"/>
+      <c r="B426" s="2"/>
       <c r="C426" s="11"/>
       <c r="D426" s="11"/>
     </row>
@@ -3056,7 +3208,7 @@
       <c r="D427" s="11"/>
     </row>
     <row r="428">
-      <c r="B428" s="2"/>
+      <c r="B428" s="7"/>
       <c r="C428" s="11"/>
       <c r="D428" s="11"/>
     </row>
@@ -3096,7 +3248,7 @@
       <c r="D435" s="11"/>
     </row>
     <row r="436">
-      <c r="B436" s="7"/>
+      <c r="B436" s="12"/>
       <c r="C436" s="11"/>
       <c r="D436" s="11"/>
     </row>
@@ -3131,7 +3283,7 @@
       <c r="D442" s="11"/>
     </row>
     <row r="443">
-      <c r="B443" s="12"/>
+      <c r="B443" s="2"/>
       <c r="C443" s="11"/>
       <c r="D443" s="11"/>
     </row>
@@ -3141,7 +3293,7 @@
       <c r="D444" s="11"/>
     </row>
     <row r="445">
-      <c r="B445" s="2"/>
+      <c r="B445" s="7"/>
       <c r="C445" s="11"/>
       <c r="D445" s="11"/>
     </row>
@@ -3181,7 +3333,7 @@
       <c r="D452" s="11"/>
     </row>
     <row r="453">
-      <c r="B453" s="7"/>
+      <c r="B453" s="12"/>
       <c r="C453" s="11"/>
       <c r="D453" s="11"/>
     </row>
@@ -3216,7 +3368,7 @@
       <c r="D459" s="11"/>
     </row>
     <row r="460">
-      <c r="B460" s="12"/>
+      <c r="B460" s="2"/>
       <c r="C460" s="11"/>
       <c r="D460" s="11"/>
     </row>
@@ -3226,7 +3378,7 @@
       <c r="D461" s="11"/>
     </row>
     <row r="462">
-      <c r="B462" s="2"/>
+      <c r="B462" s="7"/>
       <c r="C462" s="11"/>
       <c r="D462" s="11"/>
     </row>
@@ -3266,7 +3418,7 @@
       <c r="D469" s="11"/>
     </row>
     <row r="470">
-      <c r="B470" s="7"/>
+      <c r="B470" s="12"/>
       <c r="C470" s="11"/>
       <c r="D470" s="11"/>
     </row>
@@ -3301,7 +3453,7 @@
       <c r="D476" s="11"/>
     </row>
     <row r="477">
-      <c r="B477" s="12"/>
+      <c r="B477" s="2"/>
       <c r="C477" s="11"/>
       <c r="D477" s="11"/>
     </row>
@@ -3311,7 +3463,7 @@
       <c r="D478" s="11"/>
     </row>
     <row r="479">
-      <c r="B479" s="2"/>
+      <c r="B479" s="7"/>
       <c r="C479" s="11"/>
       <c r="D479" s="11"/>
     </row>
@@ -3351,7 +3503,7 @@
       <c r="D486" s="11"/>
     </row>
     <row r="487">
-      <c r="B487" s="7"/>
+      <c r="B487" s="12"/>
       <c r="C487" s="11"/>
       <c r="D487" s="11"/>
     </row>
@@ -3386,7 +3538,7 @@
       <c r="D493" s="11"/>
     </row>
     <row r="494">
-      <c r="B494" s="12"/>
+      <c r="B494" s="2"/>
       <c r="C494" s="11"/>
       <c r="D494" s="11"/>
     </row>
@@ -3396,7 +3548,7 @@
       <c r="D495" s="11"/>
     </row>
     <row r="496">
-      <c r="B496" s="2"/>
+      <c r="B496" s="7"/>
       <c r="C496" s="11"/>
       <c r="D496" s="11"/>
     </row>
@@ -3436,7 +3588,7 @@
       <c r="D503" s="11"/>
     </row>
     <row r="504">
-      <c r="B504" s="7"/>
+      <c r="B504" s="12"/>
       <c r="C504" s="11"/>
       <c r="D504" s="11"/>
     </row>
@@ -3471,7 +3623,7 @@
       <c r="D510" s="11"/>
     </row>
     <row r="511">
-      <c r="B511" s="12"/>
+      <c r="B511" s="2"/>
       <c r="C511" s="11"/>
       <c r="D511" s="11"/>
     </row>
@@ -3481,7 +3633,7 @@
       <c r="D512" s="11"/>
     </row>
     <row r="513">
-      <c r="B513" s="2"/>
+      <c r="B513" s="7"/>
       <c r="C513" s="11"/>
       <c r="D513" s="11"/>
     </row>
@@ -3521,7 +3673,7 @@
       <c r="D520" s="11"/>
     </row>
     <row r="521">
-      <c r="B521" s="7"/>
+      <c r="B521" s="12"/>
       <c r="C521" s="11"/>
       <c r="D521" s="11"/>
     </row>
@@ -3556,7 +3708,7 @@
       <c r="D527" s="11"/>
     </row>
     <row r="528">
-      <c r="B528" s="12"/>
+      <c r="B528" s="2"/>
       <c r="C528" s="11"/>
       <c r="D528" s="11"/>
     </row>
@@ -3566,7 +3718,7 @@
       <c r="D529" s="11"/>
     </row>
     <row r="530">
-      <c r="B530" s="2"/>
+      <c r="B530" s="7"/>
       <c r="C530" s="11"/>
       <c r="D530" s="11"/>
     </row>
@@ -3606,7 +3758,7 @@
       <c r="D537" s="11"/>
     </row>
     <row r="538">
-      <c r="B538" s="7"/>
+      <c r="B538" s="12"/>
       <c r="C538" s="11"/>
       <c r="D538" s="11"/>
     </row>
@@ -3641,7 +3793,7 @@
       <c r="D544" s="11"/>
     </row>
     <row r="545">
-      <c r="B545" s="12"/>
+      <c r="B545" s="2"/>
       <c r="C545" s="11"/>
       <c r="D545" s="11"/>
     </row>
@@ -3651,7 +3803,7 @@
       <c r="D546" s="11"/>
     </row>
     <row r="547">
-      <c r="B547" s="2"/>
+      <c r="B547" s="7"/>
       <c r="C547" s="11"/>
       <c r="D547" s="11"/>
     </row>
@@ -3691,7 +3843,7 @@
       <c r="D554" s="11"/>
     </row>
     <row r="555">
-      <c r="B555" s="7"/>
+      <c r="B555" s="12"/>
       <c r="C555" s="11"/>
       <c r="D555" s="11"/>
     </row>
@@ -3726,7 +3878,7 @@
       <c r="D561" s="11"/>
     </row>
     <row r="562">
-      <c r="B562" s="12"/>
+      <c r="B562" s="2"/>
       <c r="C562" s="11"/>
       <c r="D562" s="11"/>
     </row>
@@ -3736,7 +3888,7 @@
       <c r="D563" s="11"/>
     </row>
     <row r="564">
-      <c r="B564" s="2"/>
+      <c r="B564" s="7"/>
       <c r="C564" s="11"/>
       <c r="D564" s="11"/>
     </row>
@@ -3776,7 +3928,7 @@
       <c r="D571" s="11"/>
     </row>
     <row r="572">
-      <c r="B572" s="7"/>
+      <c r="B572" s="12"/>
       <c r="C572" s="11"/>
       <c r="D572" s="11"/>
     </row>
@@ -3811,7 +3963,7 @@
       <c r="D578" s="11"/>
     </row>
     <row r="579">
-      <c r="B579" s="12"/>
+      <c r="B579" s="2"/>
       <c r="C579" s="11"/>
       <c r="D579" s="11"/>
     </row>
@@ -3821,7 +3973,7 @@
       <c r="D580" s="11"/>
     </row>
     <row r="581">
-      <c r="B581" s="2"/>
+      <c r="B581" s="7"/>
       <c r="C581" s="11"/>
       <c r="D581" s="11"/>
     </row>
@@ -3861,7 +4013,7 @@
       <c r="D588" s="11"/>
     </row>
     <row r="589">
-      <c r="B589" s="7"/>
+      <c r="B589" s="12"/>
       <c r="C589" s="11"/>
       <c r="D589" s="11"/>
     </row>
@@ -3896,7 +4048,7 @@
       <c r="D595" s="11"/>
     </row>
     <row r="596">
-      <c r="B596" s="12"/>
+      <c r="B596" s="2"/>
       <c r="C596" s="11"/>
       <c r="D596" s="11"/>
     </row>
@@ -3906,7 +4058,7 @@
       <c r="D597" s="11"/>
     </row>
     <row r="598">
-      <c r="B598" s="2"/>
+      <c r="B598" s="7"/>
       <c r="C598" s="11"/>
       <c r="D598" s="11"/>
     </row>
@@ -3946,7 +4098,7 @@
       <c r="D605" s="11"/>
     </row>
     <row r="606">
-      <c r="B606" s="7"/>
+      <c r="B606" s="12"/>
       <c r="C606" s="11"/>
       <c r="D606" s="11"/>
     </row>
@@ -3981,7 +4133,7 @@
       <c r="D612" s="11"/>
     </row>
     <row r="613">
-      <c r="B613" s="12"/>
+      <c r="B613" s="2"/>
       <c r="C613" s="11"/>
       <c r="D613" s="11"/>
     </row>
@@ -3991,7 +4143,7 @@
       <c r="D614" s="11"/>
     </row>
     <row r="615">
-      <c r="B615" s="2"/>
+      <c r="B615" s="7"/>
       <c r="C615" s="11"/>
       <c r="D615" s="11"/>
     </row>
@@ -4031,7 +4183,7 @@
       <c r="D622" s="11"/>
     </row>
     <row r="623">
-      <c r="B623" s="7"/>
+      <c r="B623" s="12"/>
       <c r="C623" s="11"/>
       <c r="D623" s="11"/>
     </row>
@@ -4066,7 +4218,7 @@
       <c r="D629" s="11"/>
     </row>
     <row r="630">
-      <c r="B630" s="12"/>
+      <c r="B630" s="2"/>
       <c r="C630" s="11"/>
       <c r="D630" s="11"/>
     </row>
@@ -4076,7 +4228,7 @@
       <c r="D631" s="11"/>
     </row>
     <row r="632">
-      <c r="B632" s="2"/>
+      <c r="B632" s="7"/>
       <c r="C632" s="11"/>
       <c r="D632" s="11"/>
     </row>
@@ -4116,7 +4268,7 @@
       <c r="D639" s="11"/>
     </row>
     <row r="640">
-      <c r="B640" s="7"/>
+      <c r="B640" s="12"/>
       <c r="C640" s="11"/>
       <c r="D640" s="11"/>
     </row>
@@ -4151,7 +4303,7 @@
       <c r="D646" s="11"/>
     </row>
     <row r="647">
-      <c r="B647" s="12"/>
+      <c r="B647" s="2"/>
       <c r="C647" s="11"/>
       <c r="D647" s="11"/>
     </row>
@@ -4161,7 +4313,7 @@
       <c r="D648" s="11"/>
     </row>
     <row r="649">
-      <c r="B649" s="2"/>
+      <c r="B649" s="7"/>
       <c r="C649" s="11"/>
       <c r="D649" s="11"/>
     </row>
@@ -4201,7 +4353,7 @@
       <c r="D656" s="11"/>
     </row>
     <row r="657">
-      <c r="B657" s="7"/>
+      <c r="B657" s="12"/>
       <c r="C657" s="11"/>
       <c r="D657" s="11"/>
     </row>
@@ -4236,7 +4388,7 @@
       <c r="D663" s="11"/>
     </row>
     <row r="664">
-      <c r="B664" s="12"/>
+      <c r="B664" s="2"/>
       <c r="C664" s="11"/>
       <c r="D664" s="11"/>
     </row>
@@ -4246,7 +4398,7 @@
       <c r="D665" s="11"/>
     </row>
     <row r="666">
-      <c r="B666" s="2"/>
+      <c r="B666" s="7"/>
       <c r="C666" s="11"/>
       <c r="D666" s="11"/>
     </row>
@@ -4286,7 +4438,7 @@
       <c r="D673" s="11"/>
     </row>
     <row r="674">
-      <c r="B674" s="7"/>
+      <c r="B674" s="12"/>
       <c r="C674" s="11"/>
       <c r="D674" s="11"/>
     </row>
@@ -4321,7 +4473,7 @@
       <c r="D680" s="11"/>
     </row>
     <row r="681">
-      <c r="B681" s="12"/>
+      <c r="B681" s="2"/>
       <c r="C681" s="11"/>
       <c r="D681" s="11"/>
     </row>
@@ -4331,7 +4483,7 @@
       <c r="D682" s="11"/>
     </row>
     <row r="683">
-      <c r="B683" s="2"/>
+      <c r="B683" s="7"/>
       <c r="C683" s="11"/>
       <c r="D683" s="11"/>
     </row>
@@ -4371,7 +4523,7 @@
       <c r="D690" s="11"/>
     </row>
     <row r="691">
-      <c r="B691" s="7"/>
+      <c r="B691" s="12"/>
       <c r="C691" s="11"/>
       <c r="D691" s="11"/>
     </row>
@@ -4406,7 +4558,7 @@
       <c r="D697" s="11"/>
     </row>
     <row r="698">
-      <c r="B698" s="12"/>
+      <c r="B698" s="2"/>
       <c r="C698" s="11"/>
       <c r="D698" s="11"/>
     </row>
@@ -4416,7 +4568,7 @@
       <c r="D699" s="11"/>
     </row>
     <row r="700">
-      <c r="B700" s="2"/>
+      <c r="B700" s="7"/>
       <c r="C700" s="11"/>
       <c r="D700" s="11"/>
     </row>
@@ -4456,7 +4608,7 @@
       <c r="D707" s="11"/>
     </row>
     <row r="708">
-      <c r="B708" s="7"/>
+      <c r="B708" s="12"/>
       <c r="C708" s="11"/>
       <c r="D708" s="11"/>
     </row>
@@ -4491,7 +4643,7 @@
       <c r="D714" s="11"/>
     </row>
     <row r="715">
-      <c r="B715" s="12"/>
+      <c r="B715" s="2"/>
       <c r="C715" s="11"/>
       <c r="D715" s="11"/>
     </row>
@@ -4501,7 +4653,7 @@
       <c r="D716" s="11"/>
     </row>
     <row r="717">
-      <c r="B717" s="2"/>
+      <c r="B717" s="7"/>
       <c r="C717" s="11"/>
       <c r="D717" s="11"/>
     </row>
@@ -4541,7 +4693,7 @@
       <c r="D724" s="11"/>
     </row>
     <row r="725">
-      <c r="B725" s="7"/>
+      <c r="B725" s="12"/>
       <c r="C725" s="11"/>
       <c r="D725" s="11"/>
     </row>
@@ -4576,7 +4728,7 @@
       <c r="D731" s="11"/>
     </row>
     <row r="732">
-      <c r="B732" s="12"/>
+      <c r="B732" s="2"/>
       <c r="C732" s="11"/>
       <c r="D732" s="11"/>
     </row>
@@ -4586,7 +4738,7 @@
       <c r="D733" s="11"/>
     </row>
     <row r="734">
-      <c r="B734" s="2"/>
+      <c r="B734" s="7"/>
       <c r="C734" s="11"/>
       <c r="D734" s="11"/>
     </row>
@@ -4626,7 +4778,7 @@
       <c r="D741" s="11"/>
     </row>
     <row r="742">
-      <c r="B742" s="7"/>
+      <c r="B742" s="12"/>
       <c r="C742" s="11"/>
       <c r="D742" s="11"/>
     </row>
@@ -4661,7 +4813,7 @@
       <c r="D748" s="11"/>
     </row>
     <row r="749">
-      <c r="B749" s="12"/>
+      <c r="B749" s="2"/>
       <c r="C749" s="11"/>
       <c r="D749" s="11"/>
     </row>
@@ -4671,7 +4823,7 @@
       <c r="D750" s="11"/>
     </row>
     <row r="751">
-      <c r="B751" s="2"/>
+      <c r="B751" s="7"/>
       <c r="C751" s="11"/>
       <c r="D751" s="11"/>
     </row>
@@ -4711,7 +4863,7 @@
       <c r="D758" s="11"/>
     </row>
     <row r="759">
-      <c r="B759" s="7"/>
+      <c r="B759" s="12"/>
       <c r="C759" s="11"/>
       <c r="D759" s="11"/>
     </row>
@@ -4746,7 +4898,7 @@
       <c r="D765" s="11"/>
     </row>
     <row r="766">
-      <c r="B766" s="12"/>
+      <c r="B766" s="2"/>
       <c r="C766" s="11"/>
       <c r="D766" s="11"/>
     </row>
@@ -4756,7 +4908,7 @@
       <c r="D767" s="11"/>
     </row>
     <row r="768">
-      <c r="B768" s="2"/>
+      <c r="B768" s="7"/>
       <c r="C768" s="11"/>
       <c r="D768" s="11"/>
     </row>
@@ -4796,7 +4948,7 @@
       <c r="D775" s="11"/>
     </row>
     <row r="776">
-      <c r="B776" s="7"/>
+      <c r="B776" s="12"/>
       <c r="C776" s="11"/>
       <c r="D776" s="11"/>
     </row>
@@ -4831,7 +4983,7 @@
       <c r="D782" s="11"/>
     </row>
     <row r="783">
-      <c r="B783" s="12"/>
+      <c r="B783" s="2"/>
       <c r="C783" s="11"/>
       <c r="D783" s="11"/>
     </row>
@@ -4841,7 +4993,7 @@
       <c r="D784" s="11"/>
     </row>
     <row r="785">
-      <c r="B785" s="2"/>
+      <c r="B785" s="7"/>
       <c r="C785" s="11"/>
       <c r="D785" s="11"/>
     </row>
@@ -4881,7 +5033,7 @@
       <c r="D792" s="11"/>
     </row>
     <row r="793">
-      <c r="B793" s="7"/>
+      <c r="B793" s="12"/>
       <c r="C793" s="11"/>
       <c r="D793" s="11"/>
     </row>
@@ -4916,7 +5068,7 @@
       <c r="D799" s="11"/>
     </row>
     <row r="800">
-      <c r="B800" s="12"/>
+      <c r="B800" s="2"/>
       <c r="C800" s="11"/>
       <c r="D800" s="11"/>
     </row>
@@ -4926,7 +5078,7 @@
       <c r="D801" s="11"/>
     </row>
     <row r="802">
-      <c r="B802" s="2"/>
+      <c r="B802" s="7"/>
       <c r="C802" s="11"/>
       <c r="D802" s="11"/>
     </row>
@@ -4966,7 +5118,7 @@
       <c r="D809" s="11"/>
     </row>
     <row r="810">
-      <c r="B810" s="7"/>
+      <c r="B810" s="12"/>
       <c r="C810" s="11"/>
       <c r="D810" s="11"/>
     </row>
@@ -5001,7 +5153,7 @@
       <c r="D816" s="11"/>
     </row>
     <row r="817">
-      <c r="B817" s="12"/>
+      <c r="B817" s="2"/>
       <c r="C817" s="11"/>
       <c r="D817" s="11"/>
     </row>
@@ -5011,7 +5163,7 @@
       <c r="D818" s="11"/>
     </row>
     <row r="819">
-      <c r="B819" s="2"/>
+      <c r="B819" s="7"/>
       <c r="C819" s="11"/>
       <c r="D819" s="11"/>
     </row>
@@ -5051,7 +5203,7 @@
       <c r="D826" s="11"/>
     </row>
     <row r="827">
-      <c r="B827" s="7"/>
+      <c r="B827" s="12"/>
       <c r="C827" s="11"/>
       <c r="D827" s="11"/>
     </row>
@@ -5086,7 +5238,7 @@
       <c r="D833" s="11"/>
     </row>
     <row r="834">
-      <c r="B834" s="12"/>
+      <c r="B834" s="2"/>
       <c r="C834" s="11"/>
       <c r="D834" s="11"/>
     </row>
@@ -5096,7 +5248,7 @@
       <c r="D835" s="11"/>
     </row>
     <row r="836">
-      <c r="B836" s="2"/>
+      <c r="B836" s="7"/>
       <c r="C836" s="11"/>
       <c r="D836" s="11"/>
     </row>
@@ -5136,7 +5288,7 @@
       <c r="D843" s="11"/>
     </row>
     <row r="844">
-      <c r="B844" s="7"/>
+      <c r="B844" s="12"/>
       <c r="C844" s="11"/>
       <c r="D844" s="11"/>
     </row>
@@ -5171,7 +5323,7 @@
       <c r="D850" s="11"/>
     </row>
     <row r="851">
-      <c r="B851" s="12"/>
+      <c r="B851" s="2"/>
       <c r="C851" s="11"/>
       <c r="D851" s="11"/>
     </row>
@@ -5181,7 +5333,7 @@
       <c r="D852" s="11"/>
     </row>
     <row r="853">
-      <c r="B853" s="2"/>
+      <c r="B853" s="7"/>
       <c r="C853" s="11"/>
       <c r="D853" s="11"/>
     </row>
@@ -5221,7 +5373,7 @@
       <c r="D860" s="11"/>
     </row>
     <row r="861">
-      <c r="B861" s="7"/>
+      <c r="B861" s="12"/>
       <c r="C861" s="11"/>
       <c r="D861" s="11"/>
     </row>
@@ -5256,7 +5408,7 @@
       <c r="D867" s="11"/>
     </row>
     <row r="868">
-      <c r="B868" s="12"/>
+      <c r="B868" s="2"/>
       <c r="C868" s="11"/>
       <c r="D868" s="11"/>
     </row>
@@ -5266,7 +5418,7 @@
       <c r="D869" s="11"/>
     </row>
     <row r="870">
-      <c r="B870" s="2"/>
+      <c r="B870" s="7"/>
       <c r="C870" s="11"/>
       <c r="D870" s="11"/>
     </row>
@@ -5306,7 +5458,7 @@
       <c r="D877" s="11"/>
     </row>
     <row r="878">
-      <c r="B878" s="7"/>
+      <c r="B878" s="12"/>
       <c r="C878" s="11"/>
       <c r="D878" s="11"/>
     </row>
@@ -5341,7 +5493,7 @@
       <c r="D884" s="11"/>
     </row>
     <row r="885">
-      <c r="B885" s="12"/>
+      <c r="B885" s="2"/>
       <c r="C885" s="11"/>
       <c r="D885" s="11"/>
     </row>
@@ -5351,7 +5503,7 @@
       <c r="D886" s="11"/>
     </row>
     <row r="887">
-      <c r="B887" s="2"/>
+      <c r="B887" s="7"/>
       <c r="C887" s="11"/>
       <c r="D887" s="11"/>
     </row>
@@ -5391,7 +5543,7 @@
       <c r="D894" s="11"/>
     </row>
     <row r="895">
-      <c r="B895" s="7"/>
+      <c r="B895" s="12"/>
       <c r="C895" s="11"/>
       <c r="D895" s="11"/>
     </row>
@@ -5426,7 +5578,7 @@
       <c r="D901" s="11"/>
     </row>
     <row r="902">
-      <c r="B902" s="12"/>
+      <c r="B902" s="2"/>
       <c r="C902" s="11"/>
       <c r="D902" s="11"/>
     </row>
@@ -5436,7 +5588,7 @@
       <c r="D903" s="11"/>
     </row>
     <row r="904">
-      <c r="B904" s="2"/>
+      <c r="B904" s="7"/>
       <c r="C904" s="11"/>
       <c r="D904" s="11"/>
     </row>
@@ -5476,7 +5628,7 @@
       <c r="D911" s="11"/>
     </row>
     <row r="912">
-      <c r="B912" s="7"/>
+      <c r="B912" s="12"/>
       <c r="C912" s="11"/>
       <c r="D912" s="11"/>
     </row>
@@ -5511,7 +5663,7 @@
       <c r="D918" s="11"/>
     </row>
     <row r="919">
-      <c r="B919" s="12"/>
+      <c r="B919" s="2"/>
       <c r="C919" s="11"/>
       <c r="D919" s="11"/>
     </row>
@@ -5521,7 +5673,7 @@
       <c r="D920" s="11"/>
     </row>
     <row r="921">
-      <c r="B921" s="2"/>
+      <c r="B921" s="7"/>
       <c r="C921" s="11"/>
       <c r="D921" s="11"/>
     </row>
@@ -5561,7 +5713,7 @@
       <c r="D928" s="11"/>
     </row>
     <row r="929">
-      <c r="B929" s="7"/>
+      <c r="B929" s="12"/>
       <c r="C929" s="11"/>
       <c r="D929" s="11"/>
     </row>
@@ -5596,7 +5748,7 @@
       <c r="D935" s="11"/>
     </row>
     <row r="936">
-      <c r="B936" s="12"/>
+      <c r="B936" s="2"/>
       <c r="C936" s="11"/>
       <c r="D936" s="11"/>
     </row>
@@ -5606,7 +5758,7 @@
       <c r="D937" s="11"/>
     </row>
     <row r="938">
-      <c r="B938" s="2"/>
+      <c r="B938" s="7"/>
       <c r="C938" s="11"/>
       <c r="D938" s="11"/>
     </row>
@@ -5646,7 +5798,7 @@
       <c r="D945" s="11"/>
     </row>
     <row r="946">
-      <c r="B946" s="7"/>
+      <c r="B946" s="12"/>
       <c r="C946" s="11"/>
       <c r="D946" s="11"/>
     </row>
@@ -5681,7 +5833,7 @@
       <c r="D952" s="11"/>
     </row>
     <row r="953">
-      <c r="B953" s="12"/>
+      <c r="B953" s="2"/>
       <c r="C953" s="11"/>
       <c r="D953" s="11"/>
     </row>
@@ -5691,7 +5843,7 @@
       <c r="D954" s="11"/>
     </row>
     <row r="955">
-      <c r="B955" s="2"/>
+      <c r="B955" s="7"/>
       <c r="C955" s="11"/>
       <c r="D955" s="11"/>
     </row>
@@ -5731,7 +5883,7 @@
       <c r="D962" s="11"/>
     </row>
     <row r="963">
-      <c r="B963" s="7"/>
+      <c r="B963" s="12"/>
       <c r="C963" s="11"/>
       <c r="D963" s="11"/>
     </row>
@@ -5766,7 +5918,7 @@
       <c r="D969" s="11"/>
     </row>
     <row r="970">
-      <c r="B970" s="12"/>
+      <c r="B970" s="2"/>
       <c r="C970" s="11"/>
       <c r="D970" s="11"/>
     </row>
@@ -5776,7 +5928,7 @@
       <c r="D971" s="11"/>
     </row>
     <row r="972">
-      <c r="B972" s="2"/>
+      <c r="B972" s="7"/>
       <c r="C972" s="11"/>
       <c r="D972" s="11"/>
     </row>
@@ -5816,7 +5968,7 @@
       <c r="D979" s="11"/>
     </row>
     <row r="980">
-      <c r="B980" s="7"/>
+      <c r="B980" s="12"/>
       <c r="C980" s="11"/>
       <c r="D980" s="11"/>
     </row>
@@ -5851,7 +6003,7 @@
       <c r="D986" s="11"/>
     </row>
     <row r="987">
-      <c r="B987" s="12"/>
+      <c r="B987" s="2"/>
       <c r="C987" s="11"/>
       <c r="D987" s="11"/>
     </row>
@@ -5861,7 +6013,7 @@
       <c r="D988" s="11"/>
     </row>
     <row r="989">
-      <c r="B989" s="2"/>
+      <c r="B989" s="7"/>
       <c r="C989" s="11"/>
       <c r="D989" s="11"/>
     </row>
@@ -5901,7 +6053,7 @@
       <c r="D996" s="11"/>
     </row>
     <row r="997">
-      <c r="B997" s="7"/>
+      <c r="B997" s="12"/>
       <c r="C997" s="11"/>
       <c r="D997" s="11"/>
     </row>
@@ -5936,7 +6088,7 @@
       <c r="D1003" s="11"/>
     </row>
     <row r="1004">
-      <c r="B1004" s="12"/>
+      <c r="B1004" s="2"/>
       <c r="C1004" s="11"/>
       <c r="D1004" s="11"/>
     </row>
@@ -5946,7 +6098,7 @@
       <c r="D1005" s="11"/>
     </row>
     <row r="1006">
-      <c r="B1006" s="2"/>
+      <c r="B1006" s="7"/>
       <c r="C1006" s="11"/>
       <c r="D1006" s="11"/>
     </row>
@@ -5955,20 +6107,15 @@
       <c r="C1007" s="11"/>
       <c r="D1007" s="11"/>
     </row>
-    <row r="1008">
-      <c r="B1008" s="7"/>
-      <c r="C1008" s="11"/>
-      <c r="D1008" s="11"/>
-    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D3:D17 D19:D35 D37:D1008">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D3:D17 D19:D35 D37:D45 D47:D1007">
       <formula1>"OK,Pendiente"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C3:C17 C19:C35 C37:C1008">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C3:C17 C19:C35 C37:C45 C47:C1007">
       <formula1>"Bastian Benítez ,Eliam Rivas ,Francisco Torres ,Samir Saud,Gerónimo Lopez ,Manuel Vidal"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B3:B17 B19:B35 B37:B1008">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B3:B17 B19:B35 B37:B45 B47:B1007">
       <formula1>"Bastian Benítez ,Eliam Rivas ,Francisco Torres,Gerónimo Lopez,Manuel Vidal ,Samir Saud"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>